<commit_message>
worksheet changes for profitability
</commit_message>
<xml_diff>
--- a/banks/ACCESS BANK UK FINANCIALS.xlsx
+++ b/banks/ACCESS BANK UK FINANCIALS.xlsx
@@ -13,19 +13,20 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statement of Changes in Equity" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow Statement" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset Quality" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM1 Key Metrics" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Capital" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Ratio" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Capital" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Ratio" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital Ratio" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total RWAs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RWA Breakdown" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage Ratio" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCR" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSFR" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MREL Ratio" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Profitability" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KM1 Key Metrics" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Capital" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CET1 Ratio" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Capital" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tier 1 Ratio" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Capital Ratio" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total RWAs" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RWA Breakdown" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leverage Ratio" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCR" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NSFR" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MREL Ratio" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3279,14 +3280,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Access Bank UK Limited — Tier 1 Capital</t>
+          <t>The Access Bank UK Limited — CET1 Ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>£'000 (conv. from USD)</t>
+          <t>% of RWA</t>
         </is>
       </c>
     </row>
@@ -3330,32 +3331,44 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Tier 1 capital</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>586186</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>599900.9</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>531687.1</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>402448.5</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>279437.2</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>248093.1</v>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
+          <t>Common Equity Tier 1 (CET1) ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>11.78%</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>20.18%</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>21.88%</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>18.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: Equal to CET1 capital for FY2020-FY2024 - the Bank held no Additional Tier 1 (AT1) instruments in those years. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
+          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
         </is>
       </c>
     </row>
@@ -3423,14 +3436,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Access Bank UK Limited — Tier 1 Ratio</t>
+          <t>The Access Bank UK Limited — Tier 1 Capital</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>£'000 (conv. from USD)</t>
         </is>
       </c>
     </row>
@@ -3474,44 +3487,32 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Tier 1 ratio</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>19.27%</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>20.18%</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>22.4%</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>19.8%</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>21.88%</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>18.40%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="39" customHeight="1">
+          <t>Tier 1 capital</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>586186</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>599900.9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>531687.1</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>402448.5</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>279437.2</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>248093.1</v>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
+          <t>Note: Equal to CET1 capital for FY2020-FY2024 - the Bank held no Additional Tier 1 (AT1) instruments in those years. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
         </is>
       </c>
     </row>
@@ -3579,14 +3580,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Access Bank UK Limited — Total Capital</t>
+          <t>The Access Bank UK Limited — Tier 1 Ratio</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>£'000 (conv. from USD)</t>
+          <t>% of RWA</t>
         </is>
       </c>
     </row>
@@ -3630,32 +3631,44 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Total capital</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>586186</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>599900.9</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>531687.1</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>402448.5</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>279437.2</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>248093.1</v>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1">
+          <t>Tier 1 ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>19.27%</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>20.18%</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>21.88%</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>18.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: Equal to Tier 1 capital in every year shown, including FY2025 - the Bank's own capital-management note states in every edition that 'the Bank's regulatory capital consists only of Tier 1 capital', so it holds no Tier 2. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%. The AT1 issuance therefore splits CET1 away from Tier 1 without splitting Tier 1 away from Total capital.</t>
+          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
         </is>
       </c>
     </row>
@@ -3723,14 +3736,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Access Bank UK Limited — Total Capital Ratio</t>
+          <t>The Access Bank UK Limited — Total Capital</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>£'000 (conv. from USD)</t>
         </is>
       </c>
     </row>
@@ -3774,44 +3787,32 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Total capital ratio</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>19.27%</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>20.18%</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>22.4%</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>19.8%</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>21.88%</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>18.40%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="39" customHeight="1">
+          <t>Total capital</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>586186</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>599900.9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>531687.1</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>402448.5</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>279437.2</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>248093.1</v>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: Equal to the Tier 1 ratio in every year shown - no Tier 2 instruments. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
+          <t>Note: Equal to Tier 1 capital in every year shown, including FY2025 - the Bank's own capital-management note states in every edition that 'the Bank's regulatory capital consists only of Tier 1 capital', so it holds no Tier 2. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%. The AT1 issuance therefore splits CET1 away from Tier 1 without splitting Tier 1 away from Total capital.</t>
         </is>
       </c>
     </row>
@@ -3859,6 +3860,162 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The Access Bank UK Limited — Total Capital Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>% of RWA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Total capital ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>19.27%</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>20.18%</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>22.4%</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>19.8%</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>21.88%</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>18.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Note: Equal to the Tier 1 ratio in every year shown - no Tier 2 instruments. FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="234" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Sources - The Access Bank UK Limited Pillar 3 Disclosures (UK KM1 - Key Metrics template, or the equivalent UK CC1/LR2 tables for FY2020/FY2021 which pre-date the Bank's KM1 template), converted from USD to £ where a $ amount (see FX conversion note on the Cash Flow Statement sheet; % ratios are unconverted):
+FY2023 &amp; FY2022: Pillar 3 Disclosures 2023, p.6 (Section 1.7, Key Metrics) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/PIllar-3-2023.pdf
+FY2021 (capital/leverage): Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/10/PILLAR-3-DISCLOSURES-2021-Final.pdf
+FY2021 (LCR/NSFR) &amp; FY2020 (capital/leverage): Pillar 3 Disclosures 2022, p.6-7 (Section 1.7 comparative column) &amp; Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2024/01/PILLAR-3-DISCLOSURES-2022-Final.pdf
+FY2019: Pillar 3 Disclosures 2020, p.6 (Section 1.7 FY2019 comparative) and p.17/p.20 (Pillar 1 / leverage comparatives) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/06/PILLAR-3-DISCLOSURES-2020-Clean.pdf
+FY2025 (Tier 1 / Total capital amount): Report &amp; Financial Statements 2025, p.81, Note 28g 'Capital management', 'Capital Resources' table, Bank 31 December 2025 column - Total regulatory capital $788,303 thousand - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
+FY2025 (CET1, Tier 1 and LCR ratios): Report &amp; Financial Statements 2025, p.4, Key Performance Indicators table, Bank 2025 column - CET1 Capital Ratio 11.78%, Tier 1 Capital Ratio 19.27%, Liquidity Coverage Ratio 199.46% - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
+FY2024 (capital amounts): Report &amp; Financial Statements 2024, p.59, Note 27g 'Capital management (Bank)', 'Capital Resources' table - Total tier 1 capital / Total regulatory capital $750,775,693 (shown here as 750,776 $'000 before conversion) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/AccessBank_AR2024_Financials-AW.pdf
+SOURCE DEFECT, REPRODUCED NOT CORRECTED: the FY2025 edition's Note 28g narrative says 'Total regulatory capital as at 31 December 2025 including 2025 profit after tax was $793,036 thousand (2024: $750,776 thousand) for the Bank', while the itemised Capital Resources table immediately below it foots to $788,303 thousand (2024: $750,775). The two disagree by $4,733 thousand for 2025 and by rounding only for 2024. The TABLE figure is used here because it is the build-up the Bank shows its working for, and because the FY2024 column above was taken from the equivalent table in the previous edition; the narrative's number is recorded rather than reconciled away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="286" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>(continued)
+NO FY2024 AND NO FY2025 PILLAR 3 DISCLOSURES DOCUMENT EXISTS - and that finding is now written INTO the FY2025/FY2024 cells of KM1, Total RWAs, RWA Breakdown, Leverage Ratio, NSFR and (FY2025) CET1 Capital, not only into these notes, because a note is invisible to the coverage census and those columns otherwise read as untouched gaps. The evidence is unchanged and is set out immediately below. Independently re-confirmed a third time on 18 September 2026 in the gap-fill round: the 'Our Reports' page was re-fetched with a browser User-Agent over HTTP/1.1 (HTTP 200, text/html, 197,098 bytes), every .pdf href parsed, and it still carries exactly one Pillar 3 entry - 'Pillar 3 Disclosures 2023' at .../2025/06/PIllar-3-2023.pdf - beside 'Annual Report 2025' and 'Report and Financial Statements 2025'; a fresh Wayback CDX sweep of the domain filtered on 'pillar' still returns exactly five documents, newest the 2023 edition; and the WordPress REST media endpoint is still closed (HTTP 401, 'itsec_rest_api_access_restricted') on both /wp-json/wp/v2/media and the ?rest_route= form. Re-verified 18 September 2026 against the Bank's OWN site: its 'Our Reports' page (https://www.theaccessbankukltd.co.uk/about-us/our-reports/) carries exactly one Pillar 3 entry, 'Pillar 3 Disclosures 2023', while the same page was already carrying the FY2025 Annual Report and FY2025 Report &amp; Financial Statements - so the page is current and the Pillar 3 series is what has stopped, not our reading of it. THE PROXY IS NO LONGER NEEDED AND THE 403 IS NOT A REAL BLOCK (established 2026-09-18, second pass, and recorded because the same wrong conclusion will otherwise be drawn again): the page returns 403 to a plain curl, to curl -L, and to curl --http1.1 -L, but returns HTTP 200 with 197,459 bytes of real HTML as soon as a browser User-Agent and an Accept: text/html header are sent over HTTP/1.1. No cookie warm-up is required (one was tried and changed nothing). Cloudflare here is filtering on request HEADERS, not challenging the client. The page was re-read that way, directly from the Bank's own host with no intermediary, and every .pdf href extracted - 25 documents, of which EXACTLY ONE is a Pillar 3 ('.../2025/06/PIllar-3-2023.pdf'), alongside Annual Reports running from 2011 to 2025. That is the same result the proxy gave, now on first-hand evidence. The Bank's WordPress REST media endpoint, which would have listed unlinked uploads too, is closed (HTTP 401, 'itsec_rest_api_access_restricted'), so the reports page is the best enumeration available. A Wayback CDX sweep of the whole domain filtered on 'pillar' returns exactly five documents, the newest still the 2023 edition, and 56 further plausible 2024/2025 filenames probed under the Bank's /wp-content/uploads/ CDN (2025/06, 2025/07, 2025/12, 2026/01, 2026/05, 2026/06, 2026/07 folders) all returned non-200. Three independent routes agree. Publication lag for the next look: the Bank published its FY2025 Annual Report in June 2026 (signed 23 April 2026) and its 2023 Pillar 3 in the 2025/06 folder, i.e. its Pillar 3 has been running roughly 18 months behind year-end, so a FY2024 edition would already be overdue and a FY2025 one would not be expected before mid-2027.
+For FY2024 and FY2025 the Annual Report substitutes ONLY where the basis is verified identical. The AR's capital table is the same basis as the Pillar 3: the FY2024 edition's FY2023 comparative of $676,943,850 reproduces the FY2023 Pillar 3 CET1/Tier 1/Total capital figure of 676,944 $'000 EXACTLY, and the note confirms 'the Bank's regulatory capital consists only of Tier 1 capital'. The AR's Tier 1 Capital Ratio (20.18% for FY2024) likewise ties to the Pillar 3 basis (its FY2023 figure, 22.38%, matches the workbook's 22.4%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="169" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>(continued)
+NOT substituted for FY2024 or FY2025, and left blank rather than derived: Total RWAs (neither Annual Report gives an RWA figure; back-solving $750,775,693 / 20.18% is refused because the ratio is rounded to 2dp, which spans an RWA range of roughly $3,719.5m-$3,721.3m, and the same objection applies to $788,303k / 19.27%); Leverage Ratio (neither AR discloses a leverage ratio or a leverage exposure measure - total assets is NOT the exposure measure, which includes off-balance-sheet items); and NSFR (neither AR contains a quantitative NSFR disclosure - the FY2025 edition mentions the Net Stable Funding Ratio exactly once, in a sentence saying PRA liquidity limits 'are fully met at all times', with no figure; a richness control on the same document returns 33 hits for 'cash flow' and 16 for 'total assets', so that single hit is a fact about the document, not about the extraction). ALL THREE OF THOSE NEGATIVES WERE RE-ESTABLISHED INDEPENDENTLY ON 2026-09-18 against freshly downloaded copies of AccessBank_AR2025_web.pdf (13,090,810 bytes), AccessBank_AR2025_Financials_web.pdf (2,443,676 bytes) and the FY2024 narrative edition AccessBank_AR2024-AW4-1-v2.pdf (4,689,255 bytes), all text-native. In the FY2025 Financials edition (478,570 characters extracted) the phrase 'Risk Weighted Assets' occurs only twice and both are definitional - once in the sentence defining how the Tier 1 Capital Ratio is computed, once in Note 27/28 saying the PRA sets a minimum ratio of regulatory capital to risk-weighted assets - with no RWA AMOUNT printed anywhere; 'leverage ratio' occurs not at all; and the Net Stable Funding Ratio occurs once, in the sentence about PRA liquidity limits being 'fully met at all times'. The Key Performance Indicators table (printed under 'Key Performance Indicators') gives Bank/Group RATIOS only - LCR 199.46/195.71, CET1 ratio 11.78/11.72, Tier 1 ratio 19.27/15.58 - and no denominators. FY2020 LCR/NSFR were not found in any source (narrative-only LCR in the FY2021 Pillar 3 report gives a single FY2021 point figure, no FY2020 comparative; the UK NSFR framework may not yet have covered FY2020) - left blank.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A9:G9"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3998,7 +4155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4235,7 +4392,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4412,7 +4569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4609,7 +4766,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4785,161 +4942,6 @@
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A7:F7"/>
     <mergeCell ref="A9:F9"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>The Access Bank UK Limited — MREL Ratio</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>FY2022</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>FY2020</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>FY2019</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>MREL Ratio</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2025 (text search, 2026-09-19); no FY2025 Pillar 3 exists.</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2024 (text search, 2026-09-19); no FY2024 Pillar 3 exists.</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2023 or Annual Report (text search, 2026-09-19).</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2022 or Annual Report (text search, 2026-09-19).</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2021 or Annual Report (text search, 2026-09-19).</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2020 or Annual Report (text search, 2026-09-19).</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2019 (text search, 2026-09-19); FY2020 Pillar 3 (Dec-19 comparatives) has none.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Note: No MREL disclosure (numeric or qualitative) or UK KM2 template found in any year's Pillar 3 report - not explicitly stated as an exemption, but consistent with the Bank's small size relative to typical MREL-in-scope thresholds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="234" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Sources - The Access Bank UK Limited Pillar 3 Disclosures (UK KM1 - Key Metrics template, or the equivalent UK CC1/LR2 tables for FY2020/FY2021 which pre-date the Bank's KM1 template), converted from USD to £ where a $ amount (see FX conversion note on the Cash Flow Statement sheet; % ratios are unconverted):
-FY2023 &amp; FY2022: Pillar 3 Disclosures 2023, p.6 (Section 1.7, Key Metrics) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/PIllar-3-2023.pdf
-FY2021 (capital/leverage): Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/10/PILLAR-3-DISCLOSURES-2021-Final.pdf
-FY2021 (LCR/NSFR) &amp; FY2020 (capital/leverage): Pillar 3 Disclosures 2022, p.6-7 (Section 1.7 comparative column) &amp; Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2024/01/PILLAR-3-DISCLOSURES-2022-Final.pdf
-FY2019: Pillar 3 Disclosures 2020, p.6 (Section 1.7 FY2019 comparative) and p.17/p.20 (Pillar 1 / leverage comparatives) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/06/PILLAR-3-DISCLOSURES-2020-Clean.pdf
-FY2025 (Tier 1 / Total capital amount): Report &amp; Financial Statements 2025, p.81, Note 28g 'Capital management', 'Capital Resources' table, Bank 31 December 2025 column - Total regulatory capital $788,303 thousand - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
-FY2025 (CET1, Tier 1 and LCR ratios): Report &amp; Financial Statements 2025, p.4, Key Performance Indicators table, Bank 2025 column - CET1 Capital Ratio 11.78%, Tier 1 Capital Ratio 19.27%, Liquidity Coverage Ratio 199.46% - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
-FY2024 (capital amounts): Report &amp; Financial Statements 2024, p.59, Note 27g 'Capital management (Bank)', 'Capital Resources' table - Total tier 1 capital / Total regulatory capital $750,775,693 (shown here as 750,776 $'000 before conversion) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/AccessBank_AR2024_Financials-AW.pdf
-SOURCE DEFECT, REPRODUCED NOT CORRECTED: the FY2025 edition's Note 28g narrative says 'Total regulatory capital as at 31 December 2025 including 2025 profit after tax was $793,036 thousand (2024: $750,776 thousand) for the Bank', while the itemised Capital Resources table immediately below it foots to $788,303 thousand (2024: $750,775). The two disagree by $4,733 thousand for 2025 and by rounding only for 2024. The TABLE figure is used here because it is the build-up the Bank shows its working for, and because the FY2024 column above was taken from the equivalent table in the previous edition; the narrative's number is recorded rather than reconciled away.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="403" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>(continued)
-NO FY2024 AND NO FY2025 PILLAR 3 DISCLOSURES DOCUMENT EXISTS - and that finding is now written INTO the FY2025/FY2024 cells of KM1, Total RWAs, RWA Breakdown, Leverage Ratio, NSFR and (FY2025) CET1 Capital, not only into these notes, because a note is invisible to the coverage census and those columns otherwise read as untouched gaps. The evidence is unchanged and is set out immediately below. Independently re-confirmed a third time on 18 September 2026 in the gap-fill round: the 'Our Reports' page was re-fetched with a browser User-Agent over HTTP/1.1 (HTTP 200, text/html, 197,098 bytes), every .pdf href parsed, and it still carries exactly one Pillar 3 entry - 'Pillar 3 Disclosures 2023' at .../2025/06/PIllar-3-2023.pdf - beside 'Annual Report 2025' and 'Report and Financial Statements 2025'; a fresh Wayback CDX sweep of the domain filtered on 'pillar' still returns exactly five documents, newest the 2023 edition; and the WordPress REST media endpoint is still closed (HTTP 401, 'itsec_rest_api_access_restricted') on both /wp-json/wp/v2/media and the ?rest_route= form. Re-verified 18 September 2026 against the Bank's OWN site: its 'Our Reports' page (https://www.theaccessbankukltd.co.uk/about-us/our-reports/) carries exactly one Pillar 3 entry, 'Pillar 3 Disclosures 2023', while the same page was already carrying the FY2025 Annual Report and FY2025 Report &amp; Financial Statements - so the page is current and the Pillar 3 series is what has stopped, not our reading of it. THE PROXY IS NO LONGER NEEDED AND THE 403 IS NOT A REAL BLOCK (established 2026-09-18, second pass, and recorded because the same wrong conclusion will otherwise be drawn again): the page returns 403 to a plain curl, to curl -L, and to curl --http1.1 -L, but returns HTTP 200 with 197,459 bytes of real HTML as soon as a browser User-Agent and an Accept: text/html header are sent over HTTP/1.1. No cookie warm-up is required (one was tried and changed nothing). Cloudflare here is filtering on request HEADERS, not challenging the client. The page was re-read that way, directly from the Bank's own host with no intermediary, and every .pdf href extracted - 25 documents, of which EXACTLY ONE is a Pillar 3 ('.../2025/06/PIllar-3-2023.pdf'), alongside Annual Reports running from 2011 to 2025. That is the same result the proxy gave, now on first-hand evidence. The Bank's WordPress REST media endpoint, which would have listed unlinked uploads too, is closed (HTTP 401, 'itsec_rest_api_access_restricted'), so the reports page is the best enumeration available. A Wayback CDX sweep of the whole domain filtered on 'pillar' returns exactly five documents, the newest still the 2023 edition, and 56 further plausible 2024/2025 filenames probed under the Bank's /wp-content/uploads/ CDN (2025/06, 2025/07, 2025/12, 2026/01, 2026/05, 2026/06, 2026/07 folders) all returned non-200. Three independent routes agree. Publication lag for the next look: the Bank published its FY2025 Annual Report in June 2026 (signed 23 April 2026) and its 2023 Pillar 3 in the 2025/06 folder, i.e. its Pillar 3 has been running roughly 18 months behind year-end, so a FY2024 edition would already be overdue and a FY2025 one would not be expected before mid-2027.
-For FY2024 and FY2025 the Annual Report substitutes ONLY where the basis is verified identical. The AR's capital table is the same basis as the Pillar 3: the FY2024 edition's FY2023 comparative of $676,943,850 reproduces the FY2023 Pillar 3 CET1/Tier 1/Total capital figure of 676,944 $'000 EXACTLY, and the note confirms 'the Bank's regulatory capital consists only of Tier 1 capital'. The AR's Tier 1 Capital Ratio (20.18% for FY2024) likewise ties to the Pillar 3 basis (its FY2023 figure, 22.38%, matches the workbook's 22.4%).
-NOT substituted for FY2024 or FY2025, and left blank rather than derived: Total RWAs (neither Annual Report gives an RWA figure; back-solving $750,775,693 / 20.18% is refused because the ratio is rounded to 2dp, which spans an RWA range of roughly $3,719.5m-$3,721.3m, and the same objection applies to $788,303k / 19.27%); Leverage Ratio (neither AR discloses a leverage ratio or a leverage exposure measure - total assets is NOT the exposure measure, which includes off-balance-sheet items); and NSFR (neither AR contains a quantitative NSFR disclosure - the FY2025 edition mentions the Net Stable Funding Ratio exactly once, in a sentence saying PRA liquidity limits 'are fully met at all times', with no figure; a richness control on the same document returns 33 hits for 'cash flow' and 16 for 'total assets', so that single hit is a fact about the document, not about the extraction). ALL THREE OF THOSE NEGATIVES WERE RE-ESTABLISHED INDEPENDENTLY ON 2026-09-18 against freshly downloaded copies of AccessBank_AR2025_web.pdf (13,090,810 bytes), AccessBank_AR2025_Financials_web.pdf (2,443,676 bytes) and the FY2024 narrative edition AccessBank_AR2024-AW4-1-v2.pdf (4,689,255 bytes), all text-native. In the FY2025 Financials edition (478,570 characters extracted) the phrase 'Risk Weighted Assets' occurs only twice and both are definitional - once in the sentence defining how the Tier 1 Capital Ratio is computed, once in Note 27/28 saying the PRA sets a minimum ratio of regulatory capital to risk-weighted assets - with no RWA AMOUNT printed anywhere; 'leverage ratio' occurs not at all; and the Net Stable Funding Ratio occurs once, in the sentence about PRA liquidity limits being 'fully met at all times'. The Key Performance Indicators table (printed under 'Key Performance Indicators') gives Bank/Group RATIOS only - LCR 199.46/195.71, CET1 ratio 11.78/11.72, Tier 1 ratio 19.27/15.58 - and no denominators. FY2020 LCR/NSFR were not found in any source (narrative-only LCR in the FY2021 Pillar 3 report gives a single FY2021 point figure, no FY2020 comparative; the UK NSFR framework may not yet have covered FY2020) - left blank.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5949,6 +5951,161 @@
   <mergeCells count="2">
     <mergeCell ref="A43:H43"/>
     <mergeCell ref="A45:H45"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The Access Bank UK Limited — MREL Ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>FY2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>MREL Ratio</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2025 (text search, 2026-09-19); no FY2025 Pillar 3 exists.</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2024 (text search, 2026-09-19); no FY2024 Pillar 3 exists.</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2023 or Annual Report (text search, 2026-09-19).</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2022 or Annual Report (text search, 2026-09-19).</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2021 or Annual Report (text search, 2026-09-19).</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure or KM2 in Access Bank UK Pillar 3 FY2020 or Annual Report (text search, 2026-09-19).</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Not published – no MREL figure in Access Bank UK Annual Report FY2019 (text search, 2026-09-19); FY2020 Pillar 3 (Dec-19 comparatives) has none.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Note: No MREL disclosure (numeric or qualitative) or UK KM2 template found in any year's Pillar 3 report - not explicitly stated as an exemption, but consistent with the Bank's small size relative to typical MREL-in-scope thresholds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="234" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Sources - The Access Bank UK Limited Pillar 3 Disclosures (UK KM1 - Key Metrics template, or the equivalent UK CC1/LR2 tables for FY2020/FY2021 which pre-date the Bank's KM1 template), converted from USD to £ where a $ amount (see FX conversion note on the Cash Flow Statement sheet; % ratios are unconverted):
+FY2023 &amp; FY2022: Pillar 3 Disclosures 2023, p.6 (Section 1.7, Key Metrics) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/PIllar-3-2023.pdf
+FY2021 (capital/leverage): Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/10/PILLAR-3-DISCLOSURES-2021-Final.pdf
+FY2021 (LCR/NSFR) &amp; FY2020 (capital/leverage): Pillar 3 Disclosures 2022, p.6-7 (Section 1.7 comparative column) &amp; Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2024/01/PILLAR-3-DISCLOSURES-2022-Final.pdf
+FY2019: Pillar 3 Disclosures 2020, p.6 (Section 1.7 FY2019 comparative) and p.17/p.20 (Pillar 1 / leverage comparatives) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/06/PILLAR-3-DISCLOSURES-2020-Clean.pdf
+FY2025 (Tier 1 / Total capital amount): Report &amp; Financial Statements 2025, p.81, Note 28g 'Capital management', 'Capital Resources' table, Bank 31 December 2025 column - Total regulatory capital $788,303 thousand - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
+FY2025 (CET1, Tier 1 and LCR ratios): Report &amp; Financial Statements 2025, p.4, Key Performance Indicators table, Bank 2025 column - CET1 Capital Ratio 11.78%, Tier 1 Capital Ratio 19.27%, Liquidity Coverage Ratio 199.46% - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
+FY2024 (capital amounts): Report &amp; Financial Statements 2024, p.59, Note 27g 'Capital management (Bank)', 'Capital Resources' table - Total tier 1 capital / Total regulatory capital $750,775,693 (shown here as 750,776 $'000 before conversion) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/AccessBank_AR2024_Financials-AW.pdf
+SOURCE DEFECT, REPRODUCED NOT CORRECTED: the FY2025 edition's Note 28g narrative says 'Total regulatory capital as at 31 December 2025 including 2025 profit after tax was $793,036 thousand (2024: $750,776 thousand) for the Bank', while the itemised Capital Resources table immediately below it foots to $788,303 thousand (2024: $750,775). The two disagree by $4,733 thousand for 2025 and by rounding only for 2024. The TABLE figure is used here because it is the build-up the Bank shows its working for, and because the FY2024 column above was taken from the equivalent table in the previous edition; the narrative's number is recorded rather than reconciled away.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="403" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>(continued)
+NO FY2024 AND NO FY2025 PILLAR 3 DISCLOSURES DOCUMENT EXISTS - and that finding is now written INTO the FY2025/FY2024 cells of KM1, Total RWAs, RWA Breakdown, Leverage Ratio, NSFR and (FY2025) CET1 Capital, not only into these notes, because a note is invisible to the coverage census and those columns otherwise read as untouched gaps. The evidence is unchanged and is set out immediately below. Independently re-confirmed a third time on 18 September 2026 in the gap-fill round: the 'Our Reports' page was re-fetched with a browser User-Agent over HTTP/1.1 (HTTP 200, text/html, 197,098 bytes), every .pdf href parsed, and it still carries exactly one Pillar 3 entry - 'Pillar 3 Disclosures 2023' at .../2025/06/PIllar-3-2023.pdf - beside 'Annual Report 2025' and 'Report and Financial Statements 2025'; a fresh Wayback CDX sweep of the domain filtered on 'pillar' still returns exactly five documents, newest the 2023 edition; and the WordPress REST media endpoint is still closed (HTTP 401, 'itsec_rest_api_access_restricted') on both /wp-json/wp/v2/media and the ?rest_route= form. Re-verified 18 September 2026 against the Bank's OWN site: its 'Our Reports' page (https://www.theaccessbankukltd.co.uk/about-us/our-reports/) carries exactly one Pillar 3 entry, 'Pillar 3 Disclosures 2023', while the same page was already carrying the FY2025 Annual Report and FY2025 Report &amp; Financial Statements - so the page is current and the Pillar 3 series is what has stopped, not our reading of it. THE PROXY IS NO LONGER NEEDED AND THE 403 IS NOT A REAL BLOCK (established 2026-09-18, second pass, and recorded because the same wrong conclusion will otherwise be drawn again): the page returns 403 to a plain curl, to curl -L, and to curl --http1.1 -L, but returns HTTP 200 with 197,459 bytes of real HTML as soon as a browser User-Agent and an Accept: text/html header are sent over HTTP/1.1. No cookie warm-up is required (one was tried and changed nothing). Cloudflare here is filtering on request HEADERS, not challenging the client. The page was re-read that way, directly from the Bank's own host with no intermediary, and every .pdf href extracted - 25 documents, of which EXACTLY ONE is a Pillar 3 ('.../2025/06/PIllar-3-2023.pdf'), alongside Annual Reports running from 2011 to 2025. That is the same result the proxy gave, now on first-hand evidence. The Bank's WordPress REST media endpoint, which would have listed unlinked uploads too, is closed (HTTP 401, 'itsec_rest_api_access_restricted'), so the reports page is the best enumeration available. A Wayback CDX sweep of the whole domain filtered on 'pillar' returns exactly five documents, the newest still the 2023 edition, and 56 further plausible 2024/2025 filenames probed under the Bank's /wp-content/uploads/ CDN (2025/06, 2025/07, 2025/12, 2026/01, 2026/05, 2026/06, 2026/07 folders) all returned non-200. Three independent routes agree. Publication lag for the next look: the Bank published its FY2025 Annual Report in June 2026 (signed 23 April 2026) and its 2023 Pillar 3 in the 2025/06 folder, i.e. its Pillar 3 has been running roughly 18 months behind year-end, so a FY2024 edition would already be overdue and a FY2025 one would not be expected before mid-2027.
+For FY2024 and FY2025 the Annual Report substitutes ONLY where the basis is verified identical. The AR's capital table is the same basis as the Pillar 3: the FY2024 edition's FY2023 comparative of $676,943,850 reproduces the FY2023 Pillar 3 CET1/Tier 1/Total capital figure of 676,944 $'000 EXACTLY, and the note confirms 'the Bank's regulatory capital consists only of Tier 1 capital'. The AR's Tier 1 Capital Ratio (20.18% for FY2024) likewise ties to the Pillar 3 basis (its FY2023 figure, 22.38%, matches the workbook's 22.4%).
+NOT substituted for FY2024 or FY2025, and left blank rather than derived: Total RWAs (neither Annual Report gives an RWA figure; back-solving $750,775,693 / 20.18% is refused because the ratio is rounded to 2dp, which spans an RWA range of roughly $3,719.5m-$3,721.3m, and the same objection applies to $788,303k / 19.27%); Leverage Ratio (neither AR discloses a leverage ratio or a leverage exposure measure - total assets is NOT the exposure measure, which includes off-balance-sheet items); and NSFR (neither AR contains a quantitative NSFR disclosure - the FY2025 edition mentions the Net Stable Funding Ratio exactly once, in a sentence saying PRA liquidity limits 'are fully met at all times', with no figure; a richness control on the same document returns 33 hits for 'cash flow' and 16 for 'total assets', so that single hit is a fact about the document, not about the extraction). ALL THREE OF THOSE NEGATIVES WERE RE-ESTABLISHED INDEPENDENTLY ON 2026-09-18 against freshly downloaded copies of AccessBank_AR2025_web.pdf (13,090,810 bytes), AccessBank_AR2025_Financials_web.pdf (2,443,676 bytes) and the FY2024 narrative edition AccessBank_AR2024-AW4-1-v2.pdf (4,689,255 bytes), all text-native. In the FY2025 Financials edition (478,570 characters extracted) the phrase 'Risk Weighted Assets' occurs only twice and both are definitional - once in the sentence defining how the Tier 1 Capital Ratio is computed, once in Note 27/28 saying the PRA sets a minimum ratio of regulatory capital to risk-weighted assets - with no RWA AMOUNT printed anywhere; 'leverage ratio' occurs not at all; and the Net Stable Funding Ratio occurs once, in the sentence about PRA liquidity limits being 'fully met at all times'. The Key Performance Indicators table (printed under 'Key Performance Indicators') gives Bank/Group RATIOS only - LCR 199.46/195.71, CET1 ratio 11.78/11.72, Tier 1 ratio 19.27/15.58 - and no denominators. FY2020 LCR/NSFR were not found in any source (narrative-only LCR in the FY2021 Pillar 3 report gives a single FY2021 point figure, no FY2020 comparative; the UK NSFR framework may not yet have covered FY2020) - left blank.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9437,6 +9594,300 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="63" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>The Access Bank UK Limited — Profitability</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Return on equity and return on assets in per cent, computed from this workbook's own Balance Sheet and Profit &amp; Loss sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>FY2020</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>FY2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Return on equity - average equity basis</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Return on equity - year-end equity basis</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Return on assets - average assets basis</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Return on assets - year-end assets basis</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Not computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Pre-tax return on average shareholders' equity (as published)</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>25.83%</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Not published</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="312" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Note: TWO KINDS OF FIGURE, NEVER MERGED. The rows above are not one series. The 'Return on equity/assets' rows are THIS PROJECT'S OWN ARITHMETIC on the figures printed on this workbook's statement sheets. The rows marked '(as published)' are the bank's own published ratios, quoted verbatim, each struck on the bank's own definition - which differs from bank to bank and usually from ours, most often in whether the numerator is before or after tax and whether the denominator is average, opening or year-end equity, tangible equity or required equity. They are not averaged, reconciled, or substituted for one another, and where they disagree both stand: the disagreement is the finding.
+THE BANK'S OWN DEFINITIONS, VERBATIM. Pre-tax return on average shareholders' equity: “Return on average shareholders' equity is calculated as the profit before tax for the year divided by the average of the opening and closing shareholders' funds for the year.”
+WHY TWO BASES ARE PRINTED FOR EACH RATIO, AND NEITHER IS PREFERRED. The average basis divides by the mean of the opening and closing balance and is the fairer measure of a year in which the balance sheet moved a long way; the year-end basis divides by the closing balance alone and is what most outside sources quote. Both are shown so the reader can see which question a figure answers. They are not averaged and neither is 'the' return.
+FY2019 HAS NO AVERAGE-BASIS RATIO, AND THAT IS CORRECT. An average denominator needs an opening balance, and FY2019 is the oldest column this workbook carries, so there is no prior year to open from. The blank is structural, not a missing figure. The year-end basis is shown for FY2019 because it needs only the closing balance.
+WHY SOME CELLS SAY 'NOT COMPUTED'. Every year above is marked 'Not computed' rather than given a number, and the reason is a unit problem, not a missing figure. This workbook's statement sheets print (£'000, conv. from USD): the figures were converted from the bank's reporting currency on this project's standing convention, which converts BALANCE SHEET stocks at the financial year-end SPOT rate and PROFIT AND LOSS flows at that year's AVERAGE rate - the right treatment for each statement taken on its own. A ratio struck ACROSS the two therefore divides a figure converted at one rate by a figure converted at another. Both sides are labelled in the same currency, so such a ratio looks sound and is self-consistent on every check this project runs, but it carries the whole spot-versus-average spread - on recent years a bias of roughly two per cent of the ratio, changing sign from year to year, so it distorts the trend as well as the level. The house rule is that a ratio cancels its unit only if both sides share it; where they do not, the honest output is a refusal rather than a number with a caveat attached. A reader who wants these ratios should strike them on the bank's own figures in its own reporting currency, where both sides do share a basis. (scripts/profitability_fx_basis.py records the basis verdict for every converted workbook in this corpus, and why that verdict cannot be read off the page or detected in the code.)
+FIGURES THE BANK PUBLISHED ONLY AS A LATER EDITION'S COMPARATIVE, AND WHY THEY ARE NOT IN THE CELLS ABOVE. FY2022 Pre-tax return on average shareholders' equity 13.47%. Each year's cell carries what that year's OWN annual report printed. A comparative restated in a later edition is a different claim - it may rest on a revised definition, a restated perimeter or a corrected prior figure - so it is recorded here rather than substituted into the year it refers to.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="170" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Computed by this workbook's own build script from the Profit &amp; Loss and Balance Sheet sheets of this same workbook - the Profit &amp; Loss row “profit after tax expense for the year” and the Balance Sheet rows “total equity” and “total assets”, resolved BY LABEL at build time through the shared resolver scripts/profitability_rows.py, so this sheet cannot drift from the statements it summarises. Those rows are themselves transcribed from The Access Bank UK Limited's Annual Report and Accounts for each year; see the source cells on the Balance Sheet and Profit &amp; Loss sheets for the exact document, page and table behind every input to every percentage above.
+The '(as published)' rows are quoted verbatim from The Access Bank UK Limited's own disclosures and are recorded, with the exact document, page and verification state for each, in research/profitability/published_returns.jsonl under ‘ACCESS BANK UK’.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="A11:H11"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10263,152 +10714,6 @@
   <mergeCells count="2">
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A42:G42"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>The Access Bank UK Limited — CET1 Capital</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>£'000 (conv. from USD)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>FY2025</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>FY2022</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>FY2020</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Common Equity Tier 1 (CET1) capital</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Not disclosed - no Pillar 3 edition; the Annual Report's Capital Resources table prints Tier 1 only</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>599900.9</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>531687.1</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>402448.5</v>
-      </c>
-      <c r="F4" s="6" t="n">
-        <v>279437.2</v>
-      </c>
-      <c r="G4" s="6" t="n">
-        <v>248093.1</v>
-      </c>
-    </row>
-    <row r="5" ht="65" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%. FY2025 is therefore BLANK on this sheet: the Annual Report's Capital Resources table builds to a single 'Total regulatory capital' under the heading 'Tier one capital' and prints no CET1 amount, and no FY2025 Pillar 3 edition exists. Subtracting the convertible notes from Tier 1 to manufacture a CET1 figure is refused - it would not reproduce the Bank's own 11.78% ratio and is not a disclosure the Bank made.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="234" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Sources - The Access Bank UK Limited Pillar 3 Disclosures (UK KM1 - Key Metrics template, or the equivalent UK CC1/LR2 tables for FY2020/FY2021 which pre-date the Bank's KM1 template), converted from USD to £ where a $ amount (see FX conversion note on the Cash Flow Statement sheet; % ratios are unconverted):
-FY2023 &amp; FY2022: Pillar 3 Disclosures 2023, p.6 (Section 1.7, Key Metrics) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/PIllar-3-2023.pdf
-FY2021 (capital/leverage): Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/10/PILLAR-3-DISCLOSURES-2021-Final.pdf
-FY2021 (LCR/NSFR) &amp; FY2020 (capital/leverage): Pillar 3 Disclosures 2022, p.6-7 (Section 1.7 comparative column) &amp; Pillar 3 Disclosures 2021, p.15 (UK CC1) &amp; p.21 (LR2) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2024/01/PILLAR-3-DISCLOSURES-2022-Final.pdf
-FY2019: Pillar 3 Disclosures 2020, p.6 (Section 1.7 FY2019 comparative) and p.17/p.20 (Pillar 1 / leverage comparatives) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2022/06/PILLAR-3-DISCLOSURES-2020-Clean.pdf
-FY2025 (Tier 1 / Total capital amount): Report &amp; Financial Statements 2025, p.81, Note 28g 'Capital management', 'Capital Resources' table, Bank 31 December 2025 column - Total regulatory capital $788,303 thousand - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
-FY2025 (CET1, Tier 1 and LCR ratios): Report &amp; Financial Statements 2025, p.4, Key Performance Indicators table, Bank 2025 column - CET1 Capital Ratio 11.78%, Tier 1 Capital Ratio 19.27%, Liquidity Coverage Ratio 199.46% - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2026/06/AccessBank_AR2025_Financials_web.pdf
-FY2024 (capital amounts): Report &amp; Financial Statements 2024, p.59, Note 27g 'Capital management (Bank)', 'Capital Resources' table - Total tier 1 capital / Total regulatory capital $750,775,693 (shown here as 750,776 $'000 before conversion) - https://www.theaccessbankukltd.co.uk/wp-content/uploads/2025/06/AccessBank_AR2024_Financials-AW.pdf
-SOURCE DEFECT, REPRODUCED NOT CORRECTED: the FY2025 edition's Note 28g narrative says 'Total regulatory capital as at 31 December 2025 including 2025 profit after tax was $793,036 thousand (2024: $750,776 thousand) for the Bank', while the itemised Capital Resources table immediately below it foots to $788,303 thousand (2024: $750,775). The two disagree by $4,733 thousand for 2025 and by rounding only for 2024. The TABLE figure is used here because it is the build-up the Bank shows its working for, and because the FY2024 column above was taken from the equivalent table in the previous edition; the narrative's number is recorded rather than reconciled away.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="286" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>(continued)
-NO FY2024 AND NO FY2025 PILLAR 3 DISCLOSURES DOCUMENT EXISTS - and that finding is now written INTO the FY2025/FY2024 cells of KM1, Total RWAs, RWA Breakdown, Leverage Ratio, NSFR and (FY2025) CET1 Capital, not only into these notes, because a note is invisible to the coverage census and those columns otherwise read as untouched gaps. The evidence is unchanged and is set out immediately below. Independently re-confirmed a third time on 18 September 2026 in the gap-fill round: the 'Our Reports' page was re-fetched with a browser User-Agent over HTTP/1.1 (HTTP 200, text/html, 197,098 bytes), every .pdf href parsed, and it still carries exactly one Pillar 3 entry - 'Pillar 3 Disclosures 2023' at .../2025/06/PIllar-3-2023.pdf - beside 'Annual Report 2025' and 'Report and Financial Statements 2025'; a fresh Wayback CDX sweep of the domain filtered on 'pillar' still returns exactly five documents, newest the 2023 edition; and the WordPress REST media endpoint is still closed (HTTP 401, 'itsec_rest_api_access_restricted') on both /wp-json/wp/v2/media and the ?rest_route= form. Re-verified 18 September 2026 against the Bank's OWN site: its 'Our Reports' page (https://www.theaccessbankukltd.co.uk/about-us/our-reports/) carries exactly one Pillar 3 entry, 'Pillar 3 Disclosures 2023', while the same page was already carrying the FY2025 Annual Report and FY2025 Report &amp; Financial Statements - so the page is current and the Pillar 3 series is what has stopped, not our reading of it. THE PROXY IS NO LONGER NEEDED AND THE 403 IS NOT A REAL BLOCK (established 2026-09-18, second pass, and recorded because the same wrong conclusion will otherwise be drawn again): the page returns 403 to a plain curl, to curl -L, and to curl --http1.1 -L, but returns HTTP 200 with 197,459 bytes of real HTML as soon as a browser User-Agent and an Accept: text/html header are sent over HTTP/1.1. No cookie warm-up is required (one was tried and changed nothing). Cloudflare here is filtering on request HEADERS, not challenging the client. The page was re-read that way, directly from the Bank's own host with no intermediary, and every .pdf href extracted - 25 documents, of which EXACTLY ONE is a Pillar 3 ('.../2025/06/PIllar-3-2023.pdf'), alongside Annual Reports running from 2011 to 2025. That is the same result the proxy gave, now on first-hand evidence. The Bank's WordPress REST media endpoint, which would have listed unlinked uploads too, is closed (HTTP 401, 'itsec_rest_api_access_restricted'), so the reports page is the best enumeration available. A Wayback CDX sweep of the whole domain filtered on 'pillar' returns exactly five documents, the newest still the 2023 edition, and 56 further plausible 2024/2025 filenames probed under the Bank's /wp-content/uploads/ CDN (2025/06, 2025/07, 2025/12, 2026/01, 2026/05, 2026/06, 2026/07 folders) all returned non-200. Three independent routes agree. Publication lag for the next look: the Bank published its FY2025 Annual Report in June 2026 (signed 23 April 2026) and its 2023 Pillar 3 in the 2025/06 folder, i.e. its Pillar 3 has been running roughly 18 months behind year-end, so a FY2024 edition would already be overdue and a FY2025 one would not be expected before mid-2027.
-For FY2024 and FY2025 the Annual Report substitutes ONLY where the basis is verified identical. The AR's capital table is the same basis as the Pillar 3: the FY2024 edition's FY2023 comparative of $676,943,850 reproduces the FY2023 Pillar 3 CET1/Tier 1/Total capital figure of 676,944 $'000 EXACTLY, and the note confirms 'the Bank's regulatory capital consists only of Tier 1 capital'. The AR's Tier 1 Capital Ratio (20.18% for FY2024) likewise ties to the Pillar 3 basis (its FY2023 figure, 22.38%, matches the workbook's 22.4%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="169" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>(continued)
-NOT substituted for FY2024 or FY2025, and left blank rather than derived: Total RWAs (neither Annual Report gives an RWA figure; back-solving $750,775,693 / 20.18% is refused because the ratio is rounded to 2dp, which spans an RWA range of roughly $3,719.5m-$3,721.3m, and the same objection applies to $788,303k / 19.27%); Leverage Ratio (neither AR discloses a leverage ratio or a leverage exposure measure - total assets is NOT the exposure measure, which includes off-balance-sheet items); and NSFR (neither AR contains a quantitative NSFR disclosure - the FY2025 edition mentions the Net Stable Funding Ratio exactly once, in a sentence saying PRA liquidity limits 'are fully met at all times', with no figure; a richness control on the same document returns 33 hits for 'cash flow' and 16 for 'total assets', so that single hit is a fact about the document, not about the extraction). ALL THREE OF THOSE NEGATIVES WERE RE-ESTABLISHED INDEPENDENTLY ON 2026-09-18 against freshly downloaded copies of AccessBank_AR2025_web.pdf (13,090,810 bytes), AccessBank_AR2025_Financials_web.pdf (2,443,676 bytes) and the FY2024 narrative edition AccessBank_AR2024-AW4-1-v2.pdf (4,689,255 bytes), all text-native. In the FY2025 Financials edition (478,570 characters extracted) the phrase 'Risk Weighted Assets' occurs only twice and both are definitional - once in the sentence defining how the Tier 1 Capital Ratio is computed, once in Note 27/28 saying the PRA sets a minimum ratio of regulatory capital to risk-weighted assets - with no RWA AMOUNT printed anywhere; 'leverage ratio' occurs not at all; and the Net Stable Funding Ratio occurs once, in the sentence about PRA liquidity limits being 'fully met at all times'. The Key Performance Indicators table (printed under 'Key Performance Indicators') gives Bank/Group RATIOS only - LCR 199.46/195.71, CET1 ratio 11.78/11.72, Tier 1 ratio 19.27/15.58 - and no denominators. FY2020 LCR/NSFR were not found in any source (narrative-only LCR in the FY2021 Pillar 3 report gives a single FY2021 point figure, no FY2020 comparative; the UK NSFR framework may not yet have covered FY2020) - left blank.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A9:G9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10435,14 +10740,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The Access Bank UK Limited — CET1 Ratio</t>
+          <t>The Access Bank UK Limited — CET1 Capital</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>% of RWA</t>
+          <t>£'000 (conv. from USD)</t>
         </is>
       </c>
     </row>
@@ -10486,44 +10791,34 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Common Equity Tier 1 (CET1) ratio</t>
+          <t>Common Equity Tier 1 (CET1) capital</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>11.78%</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>20.18%</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>22.4%</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>19.8%</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>21.88%</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>18.40%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="39" customHeight="1">
+          <t>Not disclosed - no Pillar 3 edition; the Annual Report's Capital Resources table prints Tier 1 only</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>599900.9</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>531687.1</v>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>402448.5</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>279437.2</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>248093.1</v>
+      </c>
+    </row>
+    <row r="5" ht="65" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%.</t>
+          <t>Note: FY2025 IS THE FIRST YEAR CET1, TIER 1 AND TOTAL CAPITAL ARE NOT THE SAME NUMBER. For FY2020-FY2024 the Bank held no AT1 and no Tier 2 instruments, so one figure served all three and all three ratios were identical. During 2025 it issued $295.0m of convertible notes, carried as a separate equity component and treated as AT1: its FY2025 capital-management note redefines capital to include 'AT1 capital', and its own KPI table prints a CET1 ratio of 11.78% against a Tier 1 ratio of 19.27%. FY2025 is therefore BLANK on this sheet: the Annual Report's Capital Resources table builds to a single 'Total regulatory capital' under the heading 'Tier one capital' and prints no CET1 amount, and no FY2025 Pillar 3 edition exists. Subtracting the convertible notes from Tier 1 to manufacture a CET1 figure is refused - it would not reproduce the Bank's own 11.78% ratio and is not a disclosure the Bank made.</t>
         </is>
       </c>
     </row>

</xml_diff>